<commit_message>
Added data collected for task 2-STM32F0
</commit_message>
<xml_diff>
--- a/Practical3/STM32F0_Task2_Data.xlsx
+++ b/Practical3/STM32F0_Task2_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/ngrmar007_myuct_ac_za/Documents/Third Year/EEE3096s-repository/EEE3096S-Group-39/Practical3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{B006F4A2-8E07-479D-A790-D971CA4F138D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45C3BC9B-2342-4682-A017-DBF9860FC073}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{B006F4A2-8E07-479D-A790-D971CA4F138D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAEB412E-AFEC-4332-9053-261AA784B582}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{C79BCD39-4858-4225-88C9-54642E139A6A}"/>
   </bookViews>
@@ -92,13 +92,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -115,6 +118,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -437,418 +444,718 @@
   <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
-    <col min="4" max="4" width="21.21875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.44140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="21.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.44140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>100</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>128</v>
       </c>
+      <c r="D2" s="1">
+        <v>3821</v>
+      </c>
+      <c r="E2" s="1">
+        <v>429284</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="1">
         <v>160</v>
       </c>
+      <c r="D3" s="1">
+        <v>5964</v>
+      </c>
+      <c r="E3" s="1">
+        <v>670125</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="1">
         <v>192</v>
       </c>
+      <c r="D4" s="1">
+        <v>8592</v>
+      </c>
+      <c r="E4" s="1">
+        <v>966199</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="2">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="1">
         <v>224</v>
       </c>
+      <c r="D5" s="1">
+        <v>11689</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1315228</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="2">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="1">
         <v>256</v>
       </c>
+      <c r="D6" s="1">
+        <v>15287</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1716594</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2">
         <v>250</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>128</v>
       </c>
+      <c r="D7" s="1">
+        <v>7804</v>
+      </c>
+      <c r="E7" s="1">
+        <v>967946</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="2">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="1">
         <v>160</v>
       </c>
+      <c r="D8" s="1">
+        <v>12184</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1511166</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="1">
         <v>192</v>
       </c>
+      <c r="D9" s="1">
+        <v>17582</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2181757</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="2">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="1">
         <v>224</v>
       </c>
+      <c r="D10" s="1">
+        <v>23896</v>
+      </c>
+      <c r="E10" s="1">
+        <v>2965729</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="2">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="1">
         <v>256</v>
       </c>
+      <c r="D11" s="1">
+        <v>31239</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3873352</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2">
         <v>500</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>128</v>
       </c>
+      <c r="D12" s="1">
+        <v>14384</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1857678</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="1">
         <v>160</v>
       </c>
+      <c r="D13" s="1">
+        <v>22456</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2900031</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="1">
         <v>192</v>
       </c>
+      <c r="D14" s="1">
+        <v>32421</v>
+      </c>
+      <c r="E14" s="1">
+        <v>4188264</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="1">
         <v>224</v>
       </c>
+      <c r="D15" s="1">
+        <v>44046</v>
+      </c>
+      <c r="E15" s="1">
+        <v>5690272</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1">
+      <c r="D16" s="1">
+        <v>57589</v>
+      </c>
+      <c r="E16" s="1">
+        <v>7436300</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2">
         <v>750</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="2">
+      <c r="D17" s="1">
+        <v>20952</v>
+      </c>
+      <c r="E17" s="1">
+        <v>2745748</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="2">
+      <c r="D18" s="1">
+        <v>32693</v>
+      </c>
+      <c r="E18" s="1">
+        <v>4284306</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="2">
+      <c r="D19" s="1">
+        <v>47230</v>
+      </c>
+      <c r="E19" s="1">
+        <v>6190623</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="2">
+      <c r="D20" s="1">
+        <v>64152</v>
+      </c>
+      <c r="E20" s="1">
+        <v>8408947</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1">
+      <c r="D21" s="1">
+        <v>83875</v>
+      </c>
+      <c r="E21" s="1">
+        <v>10990550</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2">
         <v>1000</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="2">
+      <c r="D22" s="1">
+        <v>27514</v>
+      </c>
+      <c r="E22" s="1">
+        <v>3632998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="2">
+      <c r="D23" s="1">
+        <v>42919</v>
+      </c>
+      <c r="E23" s="1">
+        <v>5667029</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="2">
+      <c r="D24" s="1">
+        <v>62018</v>
+      </c>
+      <c r="E24" s="1">
+        <v>8190158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="2">
+      <c r="D25" s="1">
+        <v>84237</v>
+      </c>
+      <c r="E25" s="1">
+        <v>11124625</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="D26" s="1">
+        <v>110118</v>
+      </c>
+      <c r="E26" s="1">
+        <v>14538990</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="2">
         <v>100</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="2">
+      <c r="D27" s="1">
+        <v>21966</v>
+      </c>
+      <c r="E27" s="1">
+        <v>429384</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="2">
+      <c r="D28" s="1">
+        <v>34646</v>
+      </c>
+      <c r="E28" s="1">
+        <v>669829</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="2">
+      <c r="D29" s="1">
+        <v>49920</v>
+      </c>
+      <c r="E29" s="1">
+        <v>966024</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="2">
+      <c r="D30" s="1">
+        <v>68089</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1314999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1">
+      <c r="D31" s="1">
+        <v>88010</v>
+      </c>
+      <c r="E31" s="1">
+        <v>1715812</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2">
         <v>250</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="2">
+      <c r="D32" s="1">
+        <v>48596</v>
+      </c>
+      <c r="E32" s="1">
+        <v>968444</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="2">
+      <c r="D33" s="1">
+        <v>76194</v>
+      </c>
+      <c r="E33" s="1">
+        <v>1509977</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="2">
+      <c r="D34" s="1">
+        <v>109996</v>
+      </c>
+      <c r="E34" s="1">
+        <v>2179882</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="2">
+      <c r="D35" s="1">
+        <v>149714</v>
+      </c>
+      <c r="E35" s="1">
+        <v>2963391</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1">
+      <c r="D36" s="1">
+        <v>194913</v>
+      </c>
+      <c r="E36" s="1">
+        <v>3873086</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2">
         <v>500</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C37" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="2">
+      <c r="D37" s="1">
+        <v>92527</v>
+      </c>
+      <c r="E37" s="1">
+        <v>1857698</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="2">
+      <c r="D38" s="1">
+        <v>144852</v>
+      </c>
+      <c r="E38" s="1">
+        <v>2898149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="2">
+      <c r="D39" s="1">
+        <v>209137</v>
+      </c>
+      <c r="E39" s="1">
+        <v>4182966</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="2">
+      <c r="D40" s="1">
+        <v>284434</v>
+      </c>
+      <c r="E40" s="1">
+        <v>5683767</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1">
+      <c r="D41" s="1">
+        <v>371558</v>
+      </c>
+      <c r="E41" s="1">
+        <v>7437312</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2">
         <v>750</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C42" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="2">
+      <c r="D42" s="1">
+        <v>136352</v>
+      </c>
+      <c r="E42" s="1">
+        <v>2744850</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="2">
+      <c r="D43" s="1">
+        <v>213241</v>
+      </c>
+      <c r="E43" s="1">
+        <v>4280860</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="2">
+      <c r="D44" s="1">
+        <v>308009</v>
+      </c>
+      <c r="E44" s="1">
+        <v>6180580</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="2">
+      <c r="D45" s="1">
+        <v>418913</v>
+      </c>
+      <c r="E45" s="1">
+        <v>8399191</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="1">
         <v>256</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1">
+      <c r="D46" s="1">
+        <v>547592</v>
+      </c>
+      <c r="E46" s="1">
+        <v>10988990</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2">
         <v>1000</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C47" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="2">
+      <c r="D47" s="1">
+        <v>180136</v>
+      </c>
+      <c r="E47" s="1">
+        <v>3631126</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="2">
+      <c r="D48" s="1">
+        <v>281535</v>
+      </c>
+      <c r="E48" s="1">
+        <v>5661614</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="1">
         <v>192</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-      <c r="C50" s="2">
+      <c r="D49" s="1">
+        <v>406780</v>
+      </c>
+      <c r="E49" s="1">
+        <v>8176148</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="1">
         <v>224</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="2">
+      <c r="D50" s="1">
+        <v>553288</v>
+      </c>
+      <c r="E50" s="1">
+        <v>11112491</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="1">
         <v>256</v>
+      </c>
+      <c r="D51" s="1">
+        <v>723349</v>
+      </c>
+      <c r="E51" s="1">
+        <v>14534966</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
     <mergeCell ref="A27:A51"/>
     <mergeCell ref="B27:B31"/>
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:B46"/>
     <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="A2:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>